<commit_message>
Ajout CISP-3 (ICPC-3) et ORPHAcode au binding Condition.code
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 9fdcce4c51489425f52714858124509061a1ec3d
</commit_message>
<xml_diff>
--- a/nr-doc-core-condition/ig/ValueSet-fr-core-vs-condition-code.xlsx
+++ b/nr-doc-core-condition/ig/ValueSet-fr-core-vs-condition-code.xlsx
@@ -11,12 +11,14 @@
     <sheet name="Include #1" r:id="rId5" sheetId="3"/>
     <sheet name="Include #2" r:id="rId6" sheetId="4"/>
     <sheet name="Include #3" r:id="rId7" sheetId="5"/>
+    <sheet name="Include #4" r:id="rId8" sheetId="6"/>
+    <sheet name="Include #5" r:id="rId9" sheetId="7"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="43">
   <si>
     <t>Property</t>
   </si>
@@ -63,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-07T15:17:25+00:00</t>
+    <t>2026-09-14T12:24:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -90,7 +92,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Identification de la condition, du problème ou du diagnostic : CIM-10, CIM-11 (Chapitre 04), CISP-2 (ICPC-2), DRC (SFMG)</t>
+    <t>Identification de la condition, du problème ou du diagnostic : CIM-10, CIM-11 (Chapitre 04), CISP-2 (ICPC-2), CISP-3 (ICPC-3), DRC (SFMG), ORPHAcode (Orphanet)</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -138,7 +140,13 @@
     <t>http://hl7.org/fhir/sid/icpc-2</t>
   </si>
   <si>
+    <t>http://terminology.hl7.org/CodeSystem/ICPC-3</t>
+  </si>
+  <si>
     <t>https://www.sfmg.fr</t>
+  </si>
+  <si>
+    <t>https://www.orpha.net</t>
   </si>
 </sst>
 </file>
@@ -578,4 +586,84 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="30.703125" customWidth="true"/>
+    <col min="2" max="2" width="50.703125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="30.703125" customWidth="true"/>
+    <col min="2" max="2" width="50.703125" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s" s="2">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>